<commit_message>
Israel gas by-field chart: only quarters all three fields report (Q1 2024 on)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XS9pXkbpAjJDvyN5GQKL1R
</commit_message>
<xml_diff>
--- a/output/Data and Chart Outputs/israel_gas_fields_quarterly.xlsx
+++ b/output/Data and Chart Outputs/israel_gas_fields_quarterly.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Units" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Chart" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Chart - Leviathan by destinatio" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Chart - Exports" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Quarterly" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Leviathan" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Tamar" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Karish YTD" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Reports" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Units" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart - Leviathan by destinatio" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart - Exports" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leviathan" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tamar" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Karish YTD" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reports" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,8 +26,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="166" formatCode="mmm/yy"/>
+    <numFmt numFmtId="165" formatCode="mmm/yy"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -67,12 +67,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -150,13 +151,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -182,22 +183,22 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="2A78D6"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <cat>
             <numRef>
-              <f>'Chart'!$A$2:$A$27</f>
+              <f>'Chart'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Chart'!$B$2:$B$27</f>
+              <f>'Chart'!$B$2:$B$11</f>
             </numRef>
           </val>
         </ser>
@@ -210,22 +211,22 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="EB6834"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <cat>
             <numRef>
-              <f>'Chart'!$A$2:$A$27</f>
+              <f>'Chart'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Chart'!$C$2:$C$27</f>
+              <f>'Chart'!$C$2:$C$11</f>
             </numRef>
           </val>
         </ser>
@@ -238,22 +239,22 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="1BAF7A"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <cat>
             <numRef>
-              <f>'Chart'!$A$2:$A$27</f>
+              <f>'Chart'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Chart'!$D$2:$D$27</f>
+              <f>'Chart'!$D$2:$D$11</f>
             </numRef>
           </val>
         </ser>
@@ -274,8 +275,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
-          <a:bodyPr rot="-2700000" vert="horz"/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-2700000" vert="horz"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -287,8 +288,8 @@
         </txPr>
         <crossAx val="100"/>
         <lblOffset val="100"/>
-        <tickLblSkip val="2"/>
-        <tickMarkSkip val="2"/>
+        <tickLblSkip val="1"/>
+        <tickMarkSkip val="1"/>
       </catAx>
       <valAx>
         <axId val="100"/>
@@ -301,8 +302,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -319,7 +320,7 @@
         <crossAx val="10"/>
       </valAx>
       <spPr>
-        <a:ln>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -333,7 +334,7 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:ln>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:noFill/>
       <a:prstDash val="solid"/>
     </a:ln>
@@ -342,13 +343,13 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -374,10 +375,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="2A78D6"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -402,10 +403,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="EB6834"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -430,10 +431,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="1BAF7A"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -466,8 +467,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
-          <a:bodyPr rot="-2700000" vert="horz"/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-2700000" vert="horz"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -493,8 +494,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -511,7 +512,7 @@
         <crossAx val="10"/>
       </valAx>
       <spPr>
-        <a:ln>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -525,7 +526,7 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:ln>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:noFill/>
       <a:prstDash val="solid"/>
     </a:ln>
@@ -534,13 +535,13 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -566,10 +567,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="2A78D6"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -594,10 +595,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="EB6834"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -622,10 +623,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="1BAF7A"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -658,8 +659,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
-          <a:bodyPr rot="-2700000" vert="horz"/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-2700000" vert="horz"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -685,8 +686,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -703,7 +704,7 @@
         <crossAx val="10"/>
       </valAx>
       <spPr>
-        <a:ln>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -717,7 +718,7 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:ln>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:noFill/>
       <a:prstDash val="solid"/>
     </a:ln>
@@ -726,7 +727,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>5</col>
@@ -741,9 +742,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -753,7 +754,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>5</col>
@@ -768,9 +769,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -780,7 +781,7 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>5</col>
@@ -795,9 +796,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1122,7 +1123,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
@@ -1137,7 +1137,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
@@ -1152,7 +1151,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
@@ -1167,7 +1165,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
@@ -1193,7 +1190,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1222,276 +1219,142 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="n">
-        <v>43831</v>
+      <c r="A2" s="5" t="n">
+        <v>45292</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6209178021978023</v>
+        <v>1.008991428571429</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1.024514373626374</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.4656883516483517</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n">
-        <v>43922</v>
+      <c r="A3" s="5" t="n">
+        <v>45383</v>
       </c>
       <c r="B3" t="n">
-        <v>0.5821104395604396</v>
+        <v>1.086606153846154</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.8770463956043956</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.5044957142857144</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n">
-        <v>44013</v>
+      <c r="A4" s="5" t="n">
+        <v>45474</v>
       </c>
       <c r="B4" t="n">
-        <v>0.8828675</v>
+        <v>1.189951847826087</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1.044086782608696</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.6525542391304348</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n">
-        <v>44105</v>
+      <c r="A5" s="5" t="n">
+        <v>45566</v>
       </c>
       <c r="B5" t="n">
-        <v>0.7293253260869565</v>
+        <v>1.036409673913044</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.9481229239130435</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.4990120652173914</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n">
-        <v>44197</v>
+      <c r="A6" s="5" t="n">
+        <v>45658</v>
       </c>
       <c r="B6" t="n">
-        <v>1.059441</v>
+        <v>1.137918111111111</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1.0241263</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.4669388111111111</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n">
-        <v>44287</v>
+      <c r="A7" s="5" t="n">
+        <v>45748</v>
       </c>
       <c r="B7" t="n">
-        <v>1.086606153846154</v>
+        <v>0.7761472527472528</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1.005110692307692</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.4268809890109891</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n">
-        <v>44378</v>
+      <c r="A8" s="5" t="n">
+        <v>45839</v>
       </c>
       <c r="B8" t="n">
+        <v>1.189951847826087</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1.036409673913044</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.6563927934782608</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>45931</v>
+      </c>
+      <c r="B9" t="n">
         <v>1.074795217391304</v>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="n">
-        <v>44470</v>
-      </c>
-      <c r="B9" t="n">
-        <v>0.9212530434782609</v>
+      <c r="C9" t="n">
+        <v>0.8252891847826086</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.614168695652174</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n">
-        <v>44562</v>
+      <c r="A10" s="5" t="n">
+        <v>46023</v>
       </c>
       <c r="B10" t="n">
-        <v>1.059441</v>
+        <v>0.7455325555555556</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1.082984133333333</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.3766901333333333</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n">
-        <v>44652</v>
+      <c r="A11" s="5" t="n">
+        <v>46113</v>
       </c>
       <c r="B11" t="n">
-        <v>1.086606153846154</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="n">
-        <v>44743</v>
-      </c>
-      <c r="B12" t="n">
-        <v>1.151566304347826</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="n">
-        <v>44835</v>
-      </c>
-      <c r="B13" t="n">
-        <v>1.113180760869565</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="n">
-        <v>44927</v>
-      </c>
-      <c r="B14" t="n">
-        <v>1.098679555555556</v>
-      </c>
-      <c r="D14" t="n">
-        <v>0.2746698888888889</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="n">
-        <v>45017</v>
-      </c>
-      <c r="B15" t="n">
-        <v>0.970184065934066</v>
-      </c>
-      <c r="D15" t="n">
-        <v>0.4268809890109891</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="n">
-        <v>45108</v>
-      </c>
-      <c r="B16" t="n">
-        <v>1.113180760869565</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="n">
-        <v>45200</v>
-      </c>
-      <c r="B17" t="n">
-        <v>1.074795217391304</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="n">
-        <v>45292</v>
-      </c>
-      <c r="B18" t="n">
-        <v>1.008991428571429</v>
-      </c>
-      <c r="C18" t="n">
-        <v>1.024514373626374</v>
-      </c>
-      <c r="D18" t="n">
-        <v>0.4656883516483517</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="n">
-        <v>45383</v>
-      </c>
-      <c r="B19" t="n">
-        <v>1.086606153846154</v>
-      </c>
-      <c r="C19" t="n">
-        <v>0.8770463956043956</v>
-      </c>
-      <c r="D19" t="n">
-        <v>0.5044957142857144</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="n">
-        <v>45474</v>
-      </c>
-      <c r="B20" t="n">
-        <v>1.189951847826087</v>
-      </c>
-      <c r="C20" t="n">
-        <v>1.044086782608696</v>
-      </c>
-      <c r="D20" t="n">
-        <v>0.6525542391304348</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="n">
-        <v>45566</v>
-      </c>
-      <c r="B21" t="n">
-        <v>1.036409673913044</v>
-      </c>
-      <c r="C21" t="n">
-        <v>0.9481229239130435</v>
-      </c>
-      <c r="D21" t="n">
-        <v>0.4990120652173914</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="n">
-        <v>45658</v>
-      </c>
-      <c r="B22" t="n">
-        <v>1.137918111111111</v>
-      </c>
-      <c r="C22" t="n">
-        <v>1.0241263</v>
-      </c>
-      <c r="D22" t="n">
-        <v>0.4669388111111111</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="n">
-        <v>45748</v>
-      </c>
-      <c r="B23" t="n">
-        <v>0.7761472527472528</v>
-      </c>
-      <c r="C23" t="n">
-        <v>1.005110692307692</v>
-      </c>
-      <c r="D23" t="n">
-        <v>0.4268809890109891</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="n">
-        <v>45839</v>
-      </c>
-      <c r="B24" t="n">
-        <v>1.189951847826087</v>
-      </c>
-      <c r="C24" t="n">
-        <v>1.036409673913044</v>
-      </c>
-      <c r="D24" t="n">
-        <v>0.6563927934782608</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="n">
-        <v>45931</v>
-      </c>
-      <c r="B25" t="n">
-        <v>1.074795217391304</v>
-      </c>
-      <c r="C25" t="n">
-        <v>0.8252891847826086</v>
-      </c>
-      <c r="D25" t="n">
-        <v>0.614168695652174</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="n">
-        <v>46023</v>
-      </c>
-      <c r="B26" t="n">
-        <v>0.7455325555555556</v>
-      </c>
-      <c r="C26" t="n">
-        <v>1.082984133333333</v>
-      </c>
-      <c r="D26" t="n">
-        <v>0.3766901333333333</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="n">
-        <v>46113</v>
-      </c>
-      <c r="B27" t="n">
         <v>1.047798791208791</v>
       </c>
-      <c r="C27" t="n">
+      <c r="C11" t="n">
         <v>1.051679527472527</v>
       </c>
-      <c r="D27" t="n">
+      <c r="D11" t="n">
         <v>0.4540461428571428</v>
       </c>
     </row>
@@ -1536,7 +1399,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="n">
+      <c r="A2" s="5" t="n">
         <v>43831</v>
       </c>
       <c r="B2" t="n">
@@ -1550,7 +1413,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n">
+      <c r="A3" s="5" t="n">
         <v>43922</v>
       </c>
       <c r="B3" t="n">
@@ -1564,7 +1427,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n">
+      <c r="A4" s="5" t="n">
         <v>44013</v>
       </c>
       <c r="B4" t="n">
@@ -1578,7 +1441,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n">
+      <c r="A5" s="5" t="n">
         <v>44105</v>
       </c>
       <c r="B5" t="n">
@@ -1592,7 +1455,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n">
+      <c r="A6" s="5" t="n">
         <v>44197</v>
       </c>
       <c r="B6" t="n">
@@ -1606,7 +1469,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n">
+      <c r="A7" s="5" t="n">
         <v>44287</v>
       </c>
       <c r="B7" t="n">
@@ -1620,7 +1483,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n">
+      <c r="A8" s="5" t="n">
         <v>44378</v>
       </c>
       <c r="B8" t="n">
@@ -1634,7 +1497,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n">
+      <c r="A9" s="5" t="n">
         <v>44470</v>
       </c>
       <c r="B9" t="n">
@@ -1648,7 +1511,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n">
+      <c r="A10" s="5" t="n">
         <v>44562</v>
       </c>
       <c r="B10" t="n">
@@ -1662,7 +1525,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n">
+      <c r="A11" s="5" t="n">
         <v>44652</v>
       </c>
       <c r="B11" t="n">
@@ -1676,7 +1539,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="n">
+      <c r="A12" s="5" t="n">
         <v>44743</v>
       </c>
       <c r="B12" t="n">
@@ -1690,7 +1553,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="n">
+      <c r="A13" s="5" t="n">
         <v>44835</v>
       </c>
       <c r="B13" t="n">
@@ -1704,7 +1567,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="n">
+      <c r="A14" s="5" t="n">
         <v>44927</v>
       </c>
       <c r="B14" t="n">
@@ -1718,7 +1581,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="n">
+      <c r="A15" s="5" t="n">
         <v>45017</v>
       </c>
       <c r="B15" t="n">
@@ -1732,7 +1595,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="n">
+      <c r="A16" s="5" t="n">
         <v>45108</v>
       </c>
       <c r="B16" t="n">
@@ -1746,7 +1609,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="n">
+      <c r="A17" s="5" t="n">
         <v>45200</v>
       </c>
       <c r="B17" t="n">
@@ -1760,7 +1623,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="n">
+      <c r="A18" s="5" t="n">
         <v>45292</v>
       </c>
       <c r="B18" t="n">
@@ -1774,7 +1637,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="n">
+      <c r="A19" s="5" t="n">
         <v>45383</v>
       </c>
       <c r="B19" t="n">
@@ -1788,7 +1651,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="n">
+      <c r="A20" s="5" t="n">
         <v>45474</v>
       </c>
       <c r="B20" t="n">
@@ -1802,7 +1665,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="n">
+      <c r="A21" s="5" t="n">
         <v>45566</v>
       </c>
       <c r="B21" t="n">
@@ -1816,7 +1679,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="n">
+      <c r="A22" s="5" t="n">
         <v>45658</v>
       </c>
       <c r="B22" t="n">
@@ -1830,7 +1693,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="n">
+      <c r="A23" s="5" t="n">
         <v>45748</v>
       </c>
       <c r="B23" t="n">
@@ -1844,7 +1707,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="n">
+      <c r="A24" s="5" t="n">
         <v>45839</v>
       </c>
       <c r="B24" t="n">
@@ -1858,7 +1721,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="n">
+      <c r="A25" s="5" t="n">
         <v>45931</v>
       </c>
       <c r="B25" t="n">
@@ -1872,7 +1735,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="n">
+      <c r="A26" s="5" t="n">
         <v>46023</v>
       </c>
       <c r="B26" t="n">
@@ -1886,7 +1749,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="n">
+      <c r="A27" s="5" t="n">
         <v>46113</v>
       </c>
       <c r="B27" t="n">
@@ -1940,7 +1803,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="n">
+      <c r="A2" s="5" t="n">
         <v>45292</v>
       </c>
       <c r="B2" t="n">
@@ -1954,7 +1817,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n">
+      <c r="A3" s="5" t="n">
         <v>45383</v>
       </c>
       <c r="B3" t="n">
@@ -1968,7 +1831,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n">
+      <c r="A4" s="5" t="n">
         <v>45474</v>
       </c>
       <c r="B4" t="n">
@@ -1982,7 +1845,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n">
+      <c r="A5" s="5" t="n">
         <v>45566</v>
       </c>
       <c r="B5" t="n">
@@ -1996,7 +1859,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n">
+      <c r="A6" s="5" t="n">
         <v>45658</v>
       </c>
       <c r="B6" t="n">
@@ -2010,7 +1873,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n">
+      <c r="A7" s="5" t="n">
         <v>45748</v>
       </c>
       <c r="B7" t="n">
@@ -2024,7 +1887,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n">
+      <c r="A8" s="5" t="n">
         <v>45839</v>
       </c>
       <c r="B8" t="n">
@@ -2038,7 +1901,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n">
+      <c r="A9" s="5" t="n">
         <v>45931</v>
       </c>
       <c r="B9" t="n">
@@ -2052,7 +1915,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n">
+      <c r="A10" s="5" t="n">
         <v>46023</v>
       </c>
       <c r="B10" t="n">
@@ -2066,7 +1929,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n">
+      <c r="A11" s="5" t="n">
         <v>46113</v>
       </c>
       <c r="B11" t="n">

</xml_diff>